<commit_message>
Sync producer mapping Excel: add new codes, fix Kapcsandy typo
- Copy updated working-folder Excel (143->144 rows, 150->151 codes)
- Fix typo: Kapscandy code -> Kapcsandy to match campaign discount code
- Add Beausejour Duffau-Lagarrosse / Duffau (was missing entirely)
- New codes added by user: BDX82, Messorio, TheMascot, Pingus,
  Gruaud, Rousseau, cdp, o'shaughnessy

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,13 +439,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:D145"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
-    <col width="31.54296875" customWidth="1" min="1" max="1"/>
-    <col width="32.54296875" customWidth="1" min="2" max="2"/>
-    <col width="21.453125" customWidth="1" min="3" max="3"/>
-    <col width="77.54296875" customWidth="1" min="4" max="6"/>
+    <col width="31.5703125" customWidth="1" min="1" max="1"/>
+    <col width="32.5703125" customWidth="1" min="2" max="2"/>
+    <col width="29.28515625" customWidth="1" min="3" max="3"/>
+    <col width="77.5703125" customWidth="1" min="4" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2910,6 +2910,198 @@
         </is>
       </c>
     </row>
+    <row r="135" ht="15" customHeight="1">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Le Macchiole</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Messorio</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Kapscandy</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Kapcsandy</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>the Mascot</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>TheMascot</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Pingus, Pingus Amelia</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Pingus</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Pingus Amelia is one product category from Pingus</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Branaire Ducru</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Branaire</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="15" customHeight="1">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Chateauneuf du Pape</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>CDP</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="15" customHeight="1">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Gruaud Larose</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Gruaud</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Rousseau chambertin mazis</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Rousseau</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>O'Shaughnessy</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>O'Shaughnessy</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>1982 Bordeaux</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BDX82</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>All Bordeaux in vintage 1982</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Beausejour Duffau-Lagarrosse</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Duffau</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix tier/region charmap encoding + sync updated mapping Excel
- Replace remaining arrow chars in tier/region print statements
  (same charmap crash that broke producer map loading earlier)
- Re-apply Kapcsandy typo fix and Duffau row (user copy overwrote)
- Sync latest Producer - Product Mapping - Copy.xlsx from user

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D145"/>
+  <dimension ref="A1:D161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -669,12 +669,12 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Schrader</t>
+          <t>Haut Brion - Blanc</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Schrader</t>
+          <t>Blanc</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
@@ -682,17 +682,21 @@
           <t>Standalone Producer</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n"/>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Blanc stands for Haut Brion Blanc series</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Haut Bailly</t>
+          <t>Schrader</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>HautBailly</t>
+          <t>Schrader</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
@@ -705,12 +709,12 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Mouton Rothschild</t>
+          <t>Haut Bailly</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>Mouton</t>
+          <t>HautBailly</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
@@ -723,12 +727,12 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Latour</t>
+          <t>Mouton Rothschild</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>Latour</t>
+          <t>Mouton</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
@@ -741,12 +745,12 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Opus One</t>
+          <t>Latour</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>OpusOne</t>
+          <t>Latour</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
@@ -759,12 +763,12 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Krug</t>
+          <t>Opus One</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Krug</t>
+          <t>OpusOne</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
@@ -777,12 +781,12 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Colgin</t>
+          <t>Krug</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Colgin</t>
+          <t>Krug</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
@@ -795,12 +799,12 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Rauzan Segla</t>
+          <t>Colgin</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>RauzanSegla</t>
+          <t>Colgin</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
@@ -813,12 +817,12 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Cheval Blanc</t>
+          <t>Rauzan Segla</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>ChevalBlanc</t>
+          <t>RauzanSegla</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
@@ -831,12 +835,12 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Screaming Eagle</t>
+          <t>Cheval Blanc</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>TheFlight</t>
+          <t>ChevalBlanc</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
@@ -844,21 +848,17 @@
           <t>Standalone Producer</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>Screaming Eagle The Flight ONLY (excludes flagship Screaming Eagle bottlings)</t>
-        </is>
-      </c>
+      <c r="D21" s="1" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Bond Matriarch</t>
+          <t>Screaming Eagle</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>Matriarch</t>
+          <t>TheFlight</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
@@ -868,19 +868,19 @@
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>Bond Matriarch ONLY (excludes flagship Bond bottlings)</t>
+          <t>Screaming Eagle The Flight ONLY (excludes flagship Screaming Eagle bottlings)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>Sassicaia</t>
+          <t>Bond Matriarch</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Stones</t>
+          <t>Matriarch</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
@@ -888,17 +888,21 @@
           <t>Standalone Producer</t>
         </is>
       </c>
-      <c r="D23" s="1" t="n"/>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>Bond Matriarch ONLY (excludes flagship Bond bottlings)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Lail</t>
+          <t>Sassicaia</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>Lail</t>
+          <t>Stones</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
@@ -911,12 +915,12 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>Guigal</t>
+          <t>Lail</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>LALA</t>
+          <t>Lail</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
@@ -929,12 +933,12 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>Ausone</t>
+          <t>Guigal</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Ausone</t>
+          <t>LALA</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
@@ -947,12 +951,12 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Dana Estates</t>
+          <t>Ausone</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Lotus</t>
+          <t>Ausone</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
@@ -965,12 +969,12 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>Ornellaia</t>
+          <t>Dana Estates</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>Ornellaia</t>
+          <t>Lotus</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
@@ -983,12 +987,12 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Abreu</t>
+          <t>Ornellaia</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>Abreu</t>
+          <t>Ornellaia</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
@@ -1001,12 +1005,12 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>Dalla Valle</t>
+          <t>Abreu</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Maya</t>
+          <t>Abreu</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
@@ -1019,12 +1023,12 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>Trotanoy</t>
+          <t>Dalla Valle</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>Trotanoy</t>
+          <t>Maya</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
@@ -1037,12 +1041,12 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>Ducru Beaucaillou</t>
+          <t>Trotanoy</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>Ducru</t>
+          <t>Trotanoy</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
@@ -1055,12 +1059,12 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>Gaja</t>
+          <t>Ducru Beaucaillou</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>Gaja</t>
+          <t>Ducru</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
@@ -1073,12 +1077,12 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Vieaux Chateau Certan</t>
+          <t>Gaja</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>VCC</t>
+          <t>Gaja</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
@@ -1091,12 +1095,12 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>Carter</t>
+          <t>Vieaux Chateau Certan</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>CarterCellars</t>
+          <t>VCC</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
@@ -1109,12 +1113,12 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>Petrus</t>
+          <t>Carter</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>PETRUS</t>
+          <t>CarterCellars</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
@@ -1127,12 +1131,12 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>Plumpjack</t>
+          <t>Petrus</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>PlumpJack</t>
+          <t>PETRUS</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
@@ -1145,12 +1149,12 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>Lokoya Winery</t>
+          <t>Plumpjack</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>ELEVATION</t>
+          <t>PlumpJack</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
@@ -1163,52 +1167,52 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>Combo - Barton + Poyferre</t>
+          <t>Lokoya Winery</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>Leoville</t>
+          <t>ELEVATION</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>Combo offer</t>
-        </is>
-      </c>
-      <c r="D39" s="1" t="inlineStr">
-        <is>
-          <t>Leoville Barton and Leoville Poyferre</t>
-        </is>
-      </c>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>La Mission Haut Brion</t>
+          <t>Combo - Barton + Poyferre</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>LaMission</t>
+          <t>Leoville</t>
         </is>
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D40" s="1" t="n"/>
+          <t>Combo offer</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>Leoville Barton and Leoville Poyferre</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>Montrose</t>
+          <t>La Mission Haut Brion</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>Montrose</t>
+          <t>LaMission</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
@@ -1221,12 +1225,12 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>d'Yquem</t>
+          <t>Montrose</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>Sauternes</t>
+          <t>Montrose</t>
         </is>
       </c>
       <c r="C42" s="1" t="inlineStr">
@@ -1239,12 +1243,12 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>La Conseillante</t>
+          <t>d'Yquem</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>Conseillante</t>
+          <t>Sauternes</t>
         </is>
       </c>
       <c r="C43" s="1" t="inlineStr">
@@ -1257,12 +1261,12 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>Scarecrow - M. Etain</t>
+          <t>La Conseillante</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>TinMan</t>
+          <t>Conseillante</t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr">
@@ -1270,61 +1274,61 @@
           <t>Standalone Producer</t>
         </is>
       </c>
-      <c r="D44" s="1" t="inlineStr">
-        <is>
-          <t>M. Etain offer ONLY (excludes flagship Scarecrow bottles)</t>
-        </is>
-      </c>
+      <c r="D44" s="1" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>Combo - Araujo + Eisele</t>
+          <t>Scarecrow - M. Etain</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>Altagracia</t>
+          <t>TinMan</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>Combo offer</t>
+          <t>Standalone Producer</t>
         </is>
       </c>
       <c r="D45" s="1" t="inlineStr">
         <is>
-          <t>Altagracia bottlings from Araujo / Eisele Vineyard</t>
+          <t>M. Etain offer ONLY (excludes flagship Scarecrow bottles)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>Figeac</t>
+          <t>Combo - Araujo + Eisele</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>Figeac</t>
+          <t>Altagracia</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="n"/>
+          <t>Combo offer</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>Altagracia bottlings from Araujo / Eisele Vineyard</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>Pichon Baron</t>
+          <t>Figeac</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>Baron</t>
+          <t>Figeac</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr">
@@ -1337,12 +1341,12 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>Bryant Family</t>
+          <t>Pichon Baron</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>BryantFam, DB4</t>
+          <t>Baron</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr">
@@ -1350,21 +1354,17 @@
           <t>Standalone Producer</t>
         </is>
       </c>
-      <c r="D48" s="1" t="inlineStr">
-        <is>
-          <t>Include Bryant Bettina</t>
-        </is>
-      </c>
+      <c r="D48" s="1" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>Spottswoode</t>
+          <t>Bryant Family</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>Spottswoode</t>
+          <t>BryantFam, DB4</t>
         </is>
       </c>
       <c r="C49" s="1" t="inlineStr">
@@ -1372,57 +1372,61 @@
           <t>Standalone Producer</t>
         </is>
       </c>
-      <c r="D49" s="1" t="n"/>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>Include Bryant Bettina</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>Other - California Whites</t>
+          <t>Spottswoode</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>SUMMER</t>
+          <t>Spottswoode</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t>Category offer</t>
-        </is>
-      </c>
-      <c r="D50" s="1" t="inlineStr">
-        <is>
-          <t>All California white wines</t>
-        </is>
-      </c>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>Ulysses</t>
+          <t>Other - California Whites</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>Ulysses</t>
+          <t>SUMMER</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D51" s="1" t="n"/>
+          <t>Category offer</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>All California white wines</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>Lafite Rothschild</t>
+          <t>Ulysses</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>Lafite</t>
+          <t>Ulysses</t>
         </is>
       </c>
       <c r="C52" s="1" t="inlineStr">
@@ -1435,12 +1439,12 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>Las Cases</t>
+          <t>Lafite Rothschild</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>LasCases</t>
+          <t>Lafite</t>
         </is>
       </c>
       <c r="C53" s="1" t="inlineStr">
@@ -1453,12 +1457,12 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>Cos d'Estournel</t>
+          <t>Las Cases</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>CosD</t>
+          <t>LasCases</t>
         </is>
       </c>
       <c r="C54" s="1" t="inlineStr">
@@ -1471,12 +1475,12 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>William Fevre</t>
+          <t>Cos d'Estournel</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>Fevre</t>
+          <t>CosD</t>
         </is>
       </c>
       <c r="C55" s="1" t="inlineStr">
@@ -1489,12 +1493,12 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>William Fevre</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>Canon</t>
+          <t>Fevre</t>
         </is>
       </c>
       <c r="C56" s="1" t="inlineStr">
@@ -1507,12 +1511,12 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>Palmer</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>Palmer</t>
+          <t>Canon</t>
         </is>
       </c>
       <c r="C57" s="1" t="inlineStr">
@@ -1525,12 +1529,12 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>Sine Qua Non</t>
+          <t>Palmer</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>SQN10, SQN</t>
+          <t>Palmer</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr">
@@ -1543,12 +1547,12 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>Caymus</t>
+          <t>Sine Qua Non</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>Caymus</t>
+          <t>SQN10, SQN</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
@@ -1561,12 +1565,12 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>Roumier</t>
+          <t>Caymus</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>Roumier</t>
+          <t>Caymus</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
@@ -1579,12 +1583,12 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>Cardinale</t>
+          <t>Roumier</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>Cardinale</t>
+          <t>Roumier</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
@@ -1597,12 +1601,12 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>Giacosa</t>
+          <t>Cardinale</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>Giacosa</t>
+          <t>Cardinale</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
@@ -1615,12 +1619,12 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>Dominus</t>
+          <t>Giacosa</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>Dominus</t>
+          <t>Giacosa</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
@@ -1633,12 +1637,12 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>Promontory</t>
+          <t>Dominus</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>Promontory</t>
+          <t>Dominus</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
@@ -1651,12 +1655,12 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>Pichon Lalande</t>
+          <t>Promontory</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>Lalande</t>
+          <t>Promontory</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
@@ -1669,12 +1673,12 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>Fingers Crossed</t>
+          <t>Pichon Lalande</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>Crossed</t>
+          <t>Lalande</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
@@ -1687,12 +1691,12 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>Realm</t>
+          <t>Fingers Crossed</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>Realm</t>
+          <t>Crossed</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
@@ -1705,12 +1709,12 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>L'Evangile</t>
+          <t>Realm</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>Evangile</t>
+          <t>Realm</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
@@ -1723,12 +1727,12 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>Continuum</t>
+          <t>L'Evangile</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>Continuum</t>
+          <t>Evangile</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
@@ -1741,12 +1745,12 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>Vega Sicilia</t>
+          <t>Continuum</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>Tempranillo</t>
+          <t>Continuum</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
@@ -1759,12 +1763,12 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>Pavie</t>
+          <t>Vega Sicilia</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>Pavie</t>
+          <t>Tempranillo</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
@@ -1777,12 +1781,12 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>Poyferre</t>
+          <t>Pavie</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>Poyferre</t>
+          <t>Pavie</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
@@ -1795,12 +1799,12 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>Branaire Ducru</t>
+          <t>Poyferre</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>Branaire</t>
+          <t>Poyferre</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
@@ -1813,12 +1817,12 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>Peter Michael</t>
+          <t>Branaire Ducru</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>ThePoppies, PARADISE</t>
+          <t>Branaire</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
@@ -1831,12 +1835,12 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>Futo</t>
+          <t>Peter Michael</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>FUTO</t>
+          <t>ThePoppies, PARADISE</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
@@ -1849,12 +1853,12 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>Solaia</t>
+          <t>Futo</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>SOLAIA</t>
+          <t>FUTO</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
@@ -1867,12 +1871,12 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>Joseph Phelps/Phelps Insignia</t>
+          <t>Solaia</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>Phelps, INSIGNIA</t>
+          <t>SOLAIA</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr">
@@ -1885,52 +1889,52 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>Other -Abandoned Cart</t>
+          <t>Joseph Phelps/Phelps Insignia</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>lastchance</t>
+          <t>Phelps, INSIGNIA</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>Automation</t>
-        </is>
-      </c>
-      <c r="D78" s="1" t="inlineStr">
-        <is>
-          <t>Last Chance abandoned cart recovery email</t>
-        </is>
-      </c>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D78" s="1" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>Clos Fourtet</t>
+          <t>Other -Abandoned Cart</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>Fourtet</t>
+          <t>lastchance</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D79" s="1" t="n"/>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="D79" s="1" t="inlineStr">
+        <is>
+          <t>Last Chance abandoned cart recovery email</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>Comando G</t>
+          <t>Clos Fourtet</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>ComandoG</t>
+          <t>Fourtet</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr">
@@ -1943,12 +1947,12 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>Lynch Bages</t>
+          <t>Comando G</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t>LynchBages</t>
+          <t>ComandoG</t>
         </is>
       </c>
       <c r="C81" s="1" t="inlineStr">
@@ -1961,52 +1965,52 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>Combo - Peter Michael + Morlet</t>
+          <t>Lynch Bages</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
         <is>
-          <t>CAWhites</t>
+          <t>LynchBages</t>
         </is>
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>combo offer</t>
-        </is>
-      </c>
-      <c r="D82" s="1" t="inlineStr">
-        <is>
-          <t>White wines only</t>
-        </is>
-      </c>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D82" s="1" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>Angelus</t>
+          <t>Combo - Peter Michael + Morlet</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
         <is>
-          <t>Angelus</t>
+          <t>CAWhites</t>
         </is>
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D83" s="1" t="n"/>
+          <t>combo offer</t>
+        </is>
+      </c>
+      <c r="D83" s="1" t="inlineStr">
+        <is>
+          <t>White wines only</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>Chapoutier</t>
+          <t>Angelus</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>Chapoutier</t>
+          <t>Angelus</t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
@@ -2019,12 +2023,12 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>Batailley</t>
+          <t>Chapoutier</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
         <is>
-          <t>Batailley</t>
+          <t>Chapoutier</t>
         </is>
       </c>
       <c r="C85" s="1" t="inlineStr">
@@ -2037,12 +2041,12 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>Penfolds Grange</t>
+          <t>Batailley</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>Penfolds</t>
+          <t>Batailley</t>
         </is>
       </c>
       <c r="C86" s="1" t="inlineStr">
@@ -2055,12 +2059,12 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>Pontet Canet</t>
+          <t>Penfolds Grange</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
         <is>
-          <t>PontetCanet</t>
+          <t>Penfolds</t>
         </is>
       </c>
       <c r="C87" s="1" t="inlineStr">
@@ -2073,12 +2077,12 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>Eisele</t>
+          <t>Pontet Canet</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>EISELE</t>
+          <t>PontetCanet</t>
         </is>
       </c>
       <c r="C88" s="1" t="inlineStr">
@@ -2091,12 +2095,12 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>Calon Segur</t>
+          <t>Eisele</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>CalonSegur</t>
+          <t>EISELE</t>
         </is>
       </c>
       <c r="C89" s="1" t="inlineStr">
@@ -2109,12 +2113,12 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>Carruades de Lafite</t>
+          <t>Calon Segur</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>Carruades</t>
+          <t>CalonSegur</t>
         </is>
       </c>
       <c r="C90" s="1" t="inlineStr">
@@ -2127,12 +2131,12 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>Scarecrow</t>
+          <t>Carruades de Lafite</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
         <is>
-          <t>Scarecrow</t>
+          <t>Carruades</t>
         </is>
       </c>
       <c r="C91" s="1" t="inlineStr">
@@ -2145,12 +2149,12 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>La Mondotte</t>
+          <t>Scarecrow</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t>Mondotte</t>
+          <t>Scarecrow</t>
         </is>
       </c>
       <c r="C92" s="1" t="inlineStr">
@@ -2163,12 +2167,12 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>Outpost</t>
+          <t>La Mondotte</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t>OUTPOST</t>
+          <t>Mondotte</t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
@@ -2181,12 +2185,12 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>Myriad</t>
+          <t>Outpost</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>Beckstoffer</t>
+          <t>OUTPOST</t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
@@ -2199,12 +2203,12 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>La Fleur Petrus</t>
+          <t>Myriad</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t>Moueix</t>
+          <t>Beckstoffer</t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
@@ -2217,12 +2221,12 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>Blankiet</t>
+          <t>La Fleur Petrus</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>Blankiet</t>
+          <t>Moueix</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
@@ -2235,12 +2239,12 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>L'Eglise Clinet</t>
+          <t>Blankiet</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t>LegliseClinet</t>
+          <t>Blankiet</t>
         </is>
       </c>
       <c r="C97" s="1" t="inlineStr">
@@ -2253,12 +2257,12 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>Beringer</t>
+          <t>L'Eglise Clinet</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
         <is>
-          <t>Beringer</t>
+          <t>LegliseClinet</t>
         </is>
       </c>
       <c r="C98" s="1" t="inlineStr">
@@ -2271,12 +2275,12 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>Masseto</t>
+          <t>Beringer</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
         <is>
-          <t>Masseto</t>
+          <t>Beringer</t>
         </is>
       </c>
       <c r="C99" s="1" t="inlineStr">
@@ -2289,12 +2293,12 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>Rinaldi</t>
+          <t>Masseto</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
         <is>
-          <t>Rinaldi</t>
+          <t>Masseto</t>
         </is>
       </c>
       <c r="C100" s="1" t="inlineStr">
@@ -2307,12 +2311,12 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>Clinet</t>
+          <t>Rinaldi</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
         <is>
-          <t>Clinet</t>
+          <t>Rinaldi</t>
         </is>
       </c>
       <c r="C101" s="1" t="inlineStr">
@@ -2325,12 +2329,12 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>Fourrier</t>
+          <t>Clinet</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
         <is>
-          <t>Fourrier</t>
+          <t>Clinet</t>
         </is>
       </c>
       <c r="C102" s="1" t="inlineStr">
@@ -2343,52 +2347,52 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>Combo - Dom Perignon + Krug</t>
+          <t>Fourrier</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
         <is>
-          <t>Bubbles</t>
+          <t>Fourrier</t>
         </is>
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>Combo offer</t>
-        </is>
-      </c>
-      <c r="D103" s="1" t="inlineStr">
-        <is>
-          <t>champagne promotion including Dom Perignon and Krug</t>
-        </is>
-      </c>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D103" s="1" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>Malescot</t>
+          <t>Combo - Dom Perignon + Krug</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
         <is>
-          <t>Malescot</t>
+          <t>Bubbles</t>
         </is>
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D104" s="1" t="n"/>
+          <t>Combo offer</t>
+        </is>
+      </c>
+      <c r="D104" s="1" t="inlineStr">
+        <is>
+          <t>champagne promotion including Dom Perignon and Krug</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>Troplong Mondot</t>
+          <t>Malescot</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t>Troplong</t>
+          <t>Malescot</t>
         </is>
       </c>
       <c r="C105" s="1" t="inlineStr">
@@ -2401,12 +2405,12 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>beychevelle</t>
+          <t>Troplong Mondot</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
         <is>
-          <t>Beychevelle</t>
+          <t>Troplong</t>
         </is>
       </c>
       <c r="C106" s="1" t="inlineStr">
@@ -2419,12 +2423,12 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>Tusk</t>
+          <t>beychevelle</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>Tusk</t>
+          <t>Beychevelle</t>
         </is>
       </c>
       <c r="C107" s="1" t="inlineStr">
@@ -2437,12 +2441,12 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>Dom Perignon</t>
+          <t>Tusk</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
         <is>
-          <t>DomP, DomPerignon</t>
+          <t>Tusk</t>
         </is>
       </c>
       <c r="C108" s="1" t="inlineStr">
@@ -2455,12 +2459,12 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>Staglin</t>
+          <t>Dom Perignon</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>Staglin</t>
+          <t>DomP, DomPerignon</t>
         </is>
       </c>
       <c r="C109" s="1" t="inlineStr">
@@ -2473,12 +2477,12 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>La Gaffeliere</t>
+          <t>Staglin</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
         <is>
-          <t>Gaffeliere</t>
+          <t>Staglin</t>
         </is>
       </c>
       <c r="C110" s="1" t="inlineStr">
@@ -2491,12 +2495,12 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>Le Petit Cheval</t>
+          <t>La Gaffeliere</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
         <is>
-          <t>PetitCheval</t>
+          <t>Gaffeliere</t>
         </is>
       </c>
       <c r="C111" s="1" t="inlineStr">
@@ -2509,52 +2513,52 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>Combo - Cantenac Brown + Brane Cantenac</t>
+          <t>Le Petit Cheval</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
         <is>
-          <t>Cantenac</t>
+          <t>PetitCheval</t>
         </is>
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>Combo offer</t>
-        </is>
-      </c>
-      <c r="D112" s="1" t="inlineStr">
-        <is>
-          <t>Cantenac Brown and Brane Cantenac</t>
-        </is>
-      </c>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D112" s="1" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>Pavie Macquin</t>
+          <t>Combo - Cantenac Brown + Brane Cantenac</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
         <is>
-          <t>Macquin</t>
+          <t>Cantenac</t>
         </is>
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D113" s="1" t="n"/>
+          <t>Combo offer</t>
+        </is>
+      </c>
+      <c r="D113" s="1" t="inlineStr">
+        <is>
+          <t>Cantenac Brown and Brane Cantenac</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>Bellevue Mondotte</t>
+          <t>Pavie Macquin</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
         <is>
-          <t>Bellevue</t>
+          <t>Macquin</t>
         </is>
       </c>
       <c r="C114" s="1" t="inlineStr">
@@ -2567,12 +2571,12 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>Bruno Clair</t>
+          <t>Bellevue Mondotte</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>BrunoClair</t>
+          <t>Bellevue</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
@@ -2585,12 +2589,12 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>Casanova di Neri</t>
+          <t>Bruno Clair</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>Casanova</t>
+          <t>BrunoClair</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
@@ -2603,12 +2607,12 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>Saxum</t>
+          <t>Casanova di Neri</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>Saxum</t>
+          <t>Casanova</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
@@ -2621,12 +2625,12 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>Pape Clement</t>
+          <t>Saxum</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>Graves</t>
+          <t>Saxum</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
@@ -2639,12 +2643,12 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>Dunn</t>
+          <t>Pape Clement</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>Dunn</t>
+          <t>Graves</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
@@ -2657,47 +2661,48 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
+          <t>Dunn</t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="inlineStr">
+        <is>
+          <t>Dunn</t>
+        </is>
+      </c>
+      <c r="C120" s="1" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D120" s="1" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
+        <is>
           <t>Domaine Leflaive</t>
         </is>
       </c>
-      <c r="B120" s="1" t="inlineStr">
+      <c r="B121" s="1" t="inlineStr">
         <is>
           <t>leflaive</t>
         </is>
       </c>
-      <c r="C120" s="1" t="inlineStr">
-        <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D120" s="1" t="n"/>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>seven stones</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>SevenStones</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
+      <c r="C121" s="1" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D121" s="1" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Cristal</t>
+          <t>seven stones</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Golden</t>
+          <t>SevenStones</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -2709,12 +2714,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Harlan Maiden</t>
+          <t>Cristal</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>MAIDEN</t>
+          <t>Golden</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2726,12 +2731,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Poggio di Sotto</t>
+          <t>Harlan Maiden</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PoggioDiSotto</t>
+          <t>MAIDEN</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -2743,12 +2748,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Marcassin</t>
+          <t>Poggio di Sotto</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Marcassin</t>
+          <t>PoggioDiSotto</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2760,12 +2765,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Chateau du Tertre</t>
+          <t>Marcassin</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TertreMargaux</t>
+          <t>Marcassin</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -2777,12 +2782,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Grand Puy Lacoste</t>
+          <t>Chateau du Tertre</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Lacoste</t>
+          <t>TertreMargaux</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -2794,12 +2799,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Arnoux Vosnee Romanee</t>
+          <t>Grand Puy Lacoste</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Arnoux</t>
+          <t>Lacoste</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -2811,12 +2816,12 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Cerbaiona Brunello</t>
+          <t>Arnoux Vosnee Romanee</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Cerbaiona</t>
+          <t>Arnoux</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -2828,12 +2833,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Lafleur</t>
+          <t>Cerbaiona Brunello</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Lafleur</t>
+          <t>Cerbaiona</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -2845,12 +2850,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Philip Togni</t>
+          <t>Lafleur</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Togni</t>
+          <t>Lafleur</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -2862,12 +2867,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Clos de Tart</t>
+          <t>Philip Togni</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Pinault</t>
+          <t>Togni</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -2879,12 +2884,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Bartolo Mascarello</t>
+          <t>Clos de Tart</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Mascarello</t>
+          <t>Pinault</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -2896,46 +2901,46 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
+          <t>Bartolo Mascarello</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Mascarello</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
           <t>Morlet</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
+      <c r="B135" t="inlineStr">
         <is>
           <t>Morlet</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="15" customHeight="1">
-      <c r="A135" t="inlineStr">
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="15" customHeight="1">
+      <c r="A136" t="inlineStr">
         <is>
           <t>Le Macchiole</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
+      <c r="B136" t="inlineStr">
         <is>
           <t>Messorio</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>Kapscandy</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>Kapcsandy</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -2947,12 +2952,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>the Mascot</t>
+          <t>Kapscandy</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>TheMascot</t>
+          <t>Kapcsandy</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -2964,51 +2969,51 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Pingus, Pingus Amelia</t>
+          <t>the Mascot</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Pingus</t>
+          <t>TheMascot</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
           <t>Standalone Producer</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>Pingus Amelia is one product category from Pingus</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
+          <t>Pingus (including Pingus Amelia)</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Pingus</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Pingus Amelia is one product category from Pingus</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
           <t>Branaire Ducru</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
+      <c r="B140" t="inlineStr">
         <is>
           <t>Branaire</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="15" customHeight="1">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>Chateauneuf du Pape</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>CDP</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3020,29 +3025,29 @@
     <row r="141" ht="15" customHeight="1">
       <c r="A141" t="inlineStr">
         <is>
+          <t>Chateauneuf du Pape</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>CDP</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="15" customHeight="1">
+      <c r="A142" t="inlineStr">
+        <is>
           <t>Gruaud Larose</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
+      <c r="B142" t="inlineStr">
         <is>
           <t>Gruaud</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Standalone Producer</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Rousseau chambertin mazis</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Rousseau</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3054,12 +3059,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>O'Shaughnessy</t>
+          <t>Rousseau chambertin mazis</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>O'Shaughnessy</t>
+          <t>Rousseau</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3071,32 +3076,304 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>1982 Bordeaux</t>
+          <t>O'Shaughnessy</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>BDX82</t>
+          <t>O'Shaughnessy</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>All Bordeaux in vintage 1982</t>
+          <t>Standalone Producer</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
+          <t>1982 Bordeaux</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>BDX82</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>All Bordeaux in vintage 1982</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Domaine Dujac</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Dujac</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="15" customHeight="1">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Levy &amp; McClellan</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>LevyMcClellan</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="15" customHeight="1">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Bonneau du Martray</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Bonneau</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Odette</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Odette</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="15" customHeight="1">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Mugnier Bonnes Mares</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Mugnier</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="15" customHeight="1">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Montelena</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Montelena</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Verite</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Verite</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Bella Oaks</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>BellaOaks</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="15" customHeight="1">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Les Forts de Latour</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>LesForts</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Millot Echezeaux</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Millot</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Burlotto</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Burlotto</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Aubert</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Aubert</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="15" customHeight="1">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Domaine Ponsot</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Ponsot</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Dyquem</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Sauteurnes</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="15" customHeight="1">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>domaine jean grivot</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>grivot</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
           <t>Beausejour Duffau-Lagarrosse</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
+      <c r="B161" t="inlineStr">
         <is>
           <t>Duffau</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
+      <c r="C161" t="inlineStr">
         <is>
           <t>Standalone Producer</t>
         </is>

</xml_diff>

<commit_message>
Sync producer mappings: Chappellet, Smith Haut Lafitte, Jaboulet, Fontodi, Cavallotto
- Discount Code Mapping: add chappellet, Hermitage->Jaboulet, Fontodi,
  Cavallotto; fix Smith Haut Lafitte code from "Haut Lafitte" to
  "HautLafitte" so it matches the campaign-name suffix.
- Product Mapping: Chappellet/Sine Qua Non under Napa (not cult wine);
  Smith Haut Lafitte under Super Second; Jaboulet/Fontodi/Cavallotto
  under Super Tuscan Producers & Others; regions populated for all.

All 5 previously-unmapped producers now resolve with tier and region.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Kapcsandy</t>
+          <t>Kapscandy</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3365,17 +3365,92 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Beausejour Duffau-Lagarrosse</t>
+          <t>Haut-Brion Blanc</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Duffau</t>
+          <t>Blanc</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
           <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Smith Haut Lafitte</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>HautLafitte</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Jaboulet</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Hermitage</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Fontodi</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Fontodi</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Standalone Producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>chappellet</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>chappellet</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Cavallotto</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Cavallotto</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 6 producer mappings: Bevan, BigDaddy, Perse, Raya, DeMay, Larcis
Discount Code Mapping (all 6):
- Bevan Cellars        / Bevan
- Holiday Sale         / BigDaddy   (bucket pseudo-producer)
- Pavie Decesse        / Perse
- Raya                 / Raya
- Certan de May        / DeMay
- Larcis Ducasse       / Larcis

Product Mapping (4 producers — Holiday Sale is a bucket, Pavie Decesse
inherits Pavie's tier/region via substring fallback):
- Bevan Cellars     -> Napa (not cult wine)    / US / California
- Raya              -> Super Second Producers  / France / Other France
- Certan de May     -> Super Second Producers  / France / Bordeaux Right Bank
- Larcis Ducasse    -> Super Second Producers  / France / Bordeaux Right Bank

Verified: all 6 codes resolve via resolve_producer + resolve_tier + resolve_region.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D167"/>
+  <dimension ref="A1:D173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -3476,6 +3476,78 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Bevan Cellars</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Bevan</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Holiday Sale</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>BigDaddy</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Pavie Decesse</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Perse</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Raya</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Raya</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Certan de May</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>DeMay</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Larcis Ducasse</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Larcis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Map 4 discount codes: NineSuns, Priorat, Meursault, Rayas
- Nine Suns / NineSuns
- Clos Erasmus / Priorat
- Mersault White burgundy / Meursault
- Rayas / Rayas (distinct from existing Raya/Raya entry)

No tier/region assigned yet for these 4 -- will show as
Untiered/Unmapped Region until added to Producer - Product Mapping.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D173"/>
+  <dimension ref="A1:D177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -3548,6 +3548,54 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Nine Suns</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>NineSuns</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Clos Erasmus</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Priorat</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Mersault White burgundy</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Meursault</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Rayas</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Rayas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Set Offer Type = standalone producer for 10 producers
Cavallotto, Bevan Cellars, Pavie Decesse, Raya, Certan de May,
Larcis Ducasse, Nine Suns, Clos Erasmus, Mersault White burgundy, Rayas.

These were previously blank (defaulting to standalone producer at load
time); now set explicitly so the Offer Type column is authoritative and
they're included in the producer drill-down.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -3475,6 +3475,11 @@
           <t>Cavallotto</t>
         </is>
       </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3487,6 +3492,11 @@
           <t>Bevan</t>
         </is>
       </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -3511,6 +3521,11 @@
           <t>Perse</t>
         </is>
       </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3523,6 +3538,11 @@
           <t>Raya</t>
         </is>
       </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3535,6 +3555,11 @@
           <t>DeMay</t>
         </is>
       </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3547,6 +3572,11 @@
           <t>Larcis</t>
         </is>
       </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3559,6 +3589,11 @@
           <t>NineSuns</t>
         </is>
       </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3571,6 +3606,11 @@
           <t>Priorat</t>
         </is>
       </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -3583,6 +3623,11 @@
           <t>Meursault</t>
         </is>
       </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -3593,6 +3638,11 @@
       <c r="B177" t="inlineStr">
         <is>
           <t>Rayas</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync repo mapping copies: pick up Unico and Dancer codes
Repo's copy of Producer - Discount Code Mapping was stale — missing
Unico (Vega Sicilia) and Dancer (Peter Michael), both already added
to the master file. Re-synced both mapping spreadsheets from master.

Unico -> Vega Sicilia (existing tier/region: Super Tuscan Producers& Others / Spain)
Dancer -> Peter Michael (existing tier/region: Napa (not cult wine) / US / California)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>Tempranillo</t>
+          <t>Unico, Tempranillo</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>ThePoppies, PARADISE</t>
+          <t>ThePoppies, PARADISE, Dancer</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add Le Dome producer mapping (code: LeDome)
- Discount Code Mapping: Le Dome / LeDome / standalone producer
- Product Mapping: Super Second Producers tier; France / Bordeaux
  Right Bank region (Le Dome is Saint-Emilion)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Discount Code Mapping - Copy.xlsx
+++ b/Producer - Discount Code Mapping - Copy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D177"/>
+  <dimension ref="A1:D178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="31.5703125" customWidth="1" min="1" max="1"/>
@@ -3646,6 +3646,23 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Le Dome</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>LeDome</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>standalone producer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>